<commit_message>
BWP Test Suite added
</commit_message>
<xml_diff>
--- a/KatalonData/BWPBootstrapData/BWPACHData.xlsx
+++ b/KatalonData/BWPBootstrapData/BWPACHData.xlsx
@@ -1,72 +1,72 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t476046\Documents\VPS-Katalon-feature-VRelay\KatalonData\BWPBootstrapData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55E1A0A7-BC18-4D8D-8BEC-EB12C7564819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr documentId="13_ncr:1_{55E1A0A7-BC18-4D8D-8BEC-EB12C7564819}" revIDLastSave="0" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="27" activeTab="30" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="30" firstSheet="27" windowHeight="12456" windowWidth="23256" xWindow="-108" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" yWindow="-108"/>
   </bookViews>
   <sheets>
-    <sheet name="PayNowCorpNoCF" sheetId="1" r:id="rId1"/>
-    <sheet name="PayNowCorpNoCFOnly" sheetId="13" r:id="rId2"/>
-    <sheet name="ACMismatchCorp" sheetId="25" r:id="rId3"/>
-    <sheet name="PayNowCorpDCF" sheetId="8" r:id="rId4"/>
-    <sheet name="PayNowCorpSCF" sheetId="7" r:id="rId5"/>
-    <sheet name="MaxAmountErrorCorp" sheetId="19" r:id="rId6"/>
-    <sheet name="MinAmountErrorCorp" sheetId="22" r:id="rId7"/>
-    <sheet name="NoModifyAmountCorp" sheetId="16" r:id="rId8"/>
-    <sheet name="PayNowCorpNoCFReqFields" sheetId="2" r:id="rId9"/>
-    <sheet name="PayNowPCNoCF" sheetId="3" r:id="rId10"/>
-    <sheet name="PayNowPCSCF" sheetId="9" r:id="rId11"/>
-    <sheet name="PayNowPCDCF" sheetId="11" r:id="rId12"/>
-    <sheet name="ACMismatchPC" sheetId="26" r:id="rId13"/>
-    <sheet name="DualCFCeilingCorp" sheetId="27" r:id="rId14"/>
-    <sheet name="DualCFCeilingPC" sheetId="28" r:id="rId15"/>
-    <sheet name="DualCFCeilingPS" sheetId="29" r:id="rId16"/>
-    <sheet name="DualCFFlatCorp" sheetId="30" r:id="rId17"/>
-    <sheet name="DualCFFlatPC" sheetId="31" r:id="rId18"/>
-    <sheet name="DualCFFlatPS" sheetId="32" r:id="rId19"/>
-    <sheet name="DualCFPercentageCorp" sheetId="33" r:id="rId20"/>
-    <sheet name="DualCFPercentagePC" sheetId="34" r:id="rId21"/>
-    <sheet name="DualCFPercentagePS" sheetId="35" r:id="rId22"/>
-    <sheet name="SingleCFCeilingCorp" sheetId="36" r:id="rId23"/>
-    <sheet name="SingleCFCeilingPS" sheetId="38" r:id="rId24"/>
-    <sheet name="SingleCFCeilingPC" sheetId="37" r:id="rId25"/>
-    <sheet name="MissingReqFieldsCorp" sheetId="45" r:id="rId26"/>
-    <sheet name="MissingReqFieldsPersonalACH" sheetId="46" r:id="rId27"/>
-    <sheet name="ModifyPaymentsCorp1" sheetId="47" r:id="rId28"/>
-    <sheet name="ModifyPaymentsCorp2" sheetId="48" r:id="rId29"/>
-    <sheet name="ModifyPaymentsPC1" sheetId="49" r:id="rId30"/>
-    <sheet name="ModifyPaymentsPC2" sheetId="50" r:id="rId31"/>
-    <sheet name="SingleCFFlatCorp" sheetId="39" r:id="rId32"/>
-    <sheet name="SingleCFFlatPC" sheetId="40" r:id="rId33"/>
-    <sheet name="SingleCFFlatPS" sheetId="41" r:id="rId34"/>
-    <sheet name="SingleCFPercentageCorp" sheetId="42" r:id="rId35"/>
-    <sheet name="SingleCFPercentagePC" sheetId="43" r:id="rId36"/>
-    <sheet name="SingleCFPercentagePS" sheetId="44" r:id="rId37"/>
-    <sheet name="PayNowPCNoCFReqFields" sheetId="4" r:id="rId38"/>
-    <sheet name="PayNowPCNoCFOnly" sheetId="14" r:id="rId39"/>
-    <sheet name="NoModifyAmountPC" sheetId="17" r:id="rId40"/>
-    <sheet name="MinAmountErrorPC" sheetId="23" r:id="rId41"/>
-    <sheet name="MaxAmountErrorPC" sheetId="20" r:id="rId42"/>
-    <sheet name="PayNowPSNoCF" sheetId="5" r:id="rId43"/>
-    <sheet name="PayNowPSSCF" sheetId="10" r:id="rId44"/>
-    <sheet name="PayNowPSDCF" sheetId="12" r:id="rId45"/>
-    <sheet name="PayNowPSNoCFOnly" sheetId="15" r:id="rId46"/>
-    <sheet name="PayNowPSNoCFReqFields" sheetId="6" r:id="rId47"/>
-    <sheet name="NoModifyAmountPS" sheetId="18" r:id="rId48"/>
-    <sheet name="MaxAmountErrorPS" sheetId="21" r:id="rId49"/>
-    <sheet name="MinAmountErrorPS" sheetId="24" r:id="rId50"/>
+    <sheet name="PayNowCorpNoCF" r:id="rId1" sheetId="1"/>
+    <sheet name="PayNowCorpNoCFOnly" r:id="rId2" sheetId="13"/>
+    <sheet name="ACMismatchCorp" r:id="rId3" sheetId="25"/>
+    <sheet name="PayNowCorpDCF" r:id="rId4" sheetId="8"/>
+    <sheet name="PayNowCorpSCF" r:id="rId5" sheetId="7"/>
+    <sheet name="MaxAmountErrorCorp" r:id="rId6" sheetId="19"/>
+    <sheet name="MinAmountErrorCorp" r:id="rId7" sheetId="22"/>
+    <sheet name="NoModifyAmountCorp" r:id="rId8" sheetId="16"/>
+    <sheet name="PayNowCorpNoCFReqFields" r:id="rId9" sheetId="2"/>
+    <sheet name="PayNowPCNoCF" r:id="rId10" sheetId="3"/>
+    <sheet name="PayNowPCSCF" r:id="rId11" sheetId="9"/>
+    <sheet name="PayNowPCDCF" r:id="rId12" sheetId="11"/>
+    <sheet name="ACMismatchPC" r:id="rId13" sheetId="26"/>
+    <sheet name="DualCFCeilingCorp" r:id="rId14" sheetId="27"/>
+    <sheet name="DualCFCeilingPC" r:id="rId15" sheetId="28"/>
+    <sheet name="DualCFCeilingPS" r:id="rId16" sheetId="29"/>
+    <sheet name="DualCFFlatCorp" r:id="rId17" sheetId="30"/>
+    <sheet name="DualCFFlatPC" r:id="rId18" sheetId="31"/>
+    <sheet name="DualCFFlatPS" r:id="rId19" sheetId="32"/>
+    <sheet name="DualCFPercentageCorp" r:id="rId20" sheetId="33"/>
+    <sheet name="DualCFPercentagePC" r:id="rId21" sheetId="34"/>
+    <sheet name="DualCFPercentagePS" r:id="rId22" sheetId="35"/>
+    <sheet name="SingleCFCeilingCorp" r:id="rId23" sheetId="36"/>
+    <sheet name="SingleCFCeilingPS" r:id="rId24" sheetId="38"/>
+    <sheet name="SingleCFCeilingPC" r:id="rId25" sheetId="37"/>
+    <sheet name="MissingReqFieldsCorp" r:id="rId26" sheetId="45"/>
+    <sheet name="MissingReqFieldsPersonalACH" r:id="rId27" sheetId="46"/>
+    <sheet name="ModifyPaymentsCorp1" r:id="rId28" sheetId="47"/>
+    <sheet name="ModifyPaymentsCorp2" r:id="rId29" sheetId="48"/>
+    <sheet name="ModifyPaymentsPC1" r:id="rId30" sheetId="49"/>
+    <sheet name="ModifyPaymentsPC2" r:id="rId31" sheetId="50"/>
+    <sheet name="SingleCFFlatCorp" r:id="rId32" sheetId="39"/>
+    <sheet name="SingleCFFlatPC" r:id="rId33" sheetId="40"/>
+    <sheet name="SingleCFFlatPS" r:id="rId34" sheetId="41"/>
+    <sheet name="SingleCFPercentageCorp" r:id="rId35" sheetId="42"/>
+    <sheet name="SingleCFPercentagePC" r:id="rId36" sheetId="43"/>
+    <sheet name="SingleCFPercentagePS" r:id="rId37" sheetId="44"/>
+    <sheet name="PayNowPCNoCFReqFields" r:id="rId38" sheetId="4"/>
+    <sheet name="PayNowPCNoCFOnly" r:id="rId39" sheetId="14"/>
+    <sheet name="NoModifyAmountPC" r:id="rId40" sheetId="17"/>
+    <sheet name="MinAmountErrorPC" r:id="rId41" sheetId="23"/>
+    <sheet name="MaxAmountErrorPC" r:id="rId42" sheetId="20"/>
+    <sheet name="PayNowPSNoCF" r:id="rId43" sheetId="5"/>
+    <sheet name="PayNowPSSCF" r:id="rId44" sheetId="10"/>
+    <sheet name="PayNowPSDCF" r:id="rId45" sheetId="12"/>
+    <sheet name="PayNowPSNoCFOnly" r:id="rId46" sheetId="15"/>
+    <sheet name="PayNowPSNoCFReqFields" r:id="rId47" sheetId="6"/>
+    <sheet name="NoModifyAmountPS" r:id="rId48" sheetId="18"/>
+    <sheet name="MaxAmountErrorPS" r:id="rId49" sheetId="21"/>
+    <sheet name="MinAmountErrorPS" r:id="rId50" sheetId="24"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1251" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2979" uniqueCount="521">
   <si>
     <t>Result</t>
   </si>
@@ -338,12 +338,1312 @@
   </si>
   <si>
     <t>8</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:02:32 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:02:45 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:03:27 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:03:38 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:03:46 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:04:03 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:04:17 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:04:27 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:06:55 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:07:23 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:07:36 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:08:06 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:08:35 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:08:49 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:09:20 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:09:53 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:10:08 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:11:56 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:12:12 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:12:37 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:13:34 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:13:54 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:14:20 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:15:24 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:15:42 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:16:05 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:19:42 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:20:36 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:21:17 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:22:19 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:22:31 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:23:18 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:23:57 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:24:07 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:24:32 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:25:08 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:25:26 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:26:11 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:26:42 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:27:29 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:27:39 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:28:18 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:28:37 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:30:27 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:31:11 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:31:16 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:32:43 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:32:48 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:33:39 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:39:41 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:40:51 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:41:03 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:42:27 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:43:34 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:43:48 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:45:15 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:46:34 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:46:50 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:55:03 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:56:26 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:57:31 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:58:53 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 01:59:57 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:01:15 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:02:23 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:03:23 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:04:49 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:09:37 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:10:53 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:11:03 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:12:01 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:13:08 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:13:26 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:14:40 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:15:36 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:17:03 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:17:13 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:18:28 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:19:52 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:20:02 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:20:53 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 02:21:58 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:06:26 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:07:26 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:10:07 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:10:32 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:10:58 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:11:51 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:12:16 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:12:40 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:19:00 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:20:43 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:21:17 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:23:44 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:25:30 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:26:07 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:28:30 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:30:16 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:32:56 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:37:17 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:38:57 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:40:33 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:43:07 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:43:45 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:45:57 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:48:48 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:50:40 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:51:25 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:52:54 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:53:37 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 16:55:30 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:06:28 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:08:14 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:08:49 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:10:26 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:11:57 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:12:41 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:14:27 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:16:04 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:18:08 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:19:54 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:22:44 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:23:20 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:25:00 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:26:38 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:27:14 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:28:56 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:29:24 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:30:48 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:31:15 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:31:38 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:32:22 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:32:45 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:33:03 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:37:44 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:39:25 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:39:49 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:43:10 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:43:42 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:44:18 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:45:28 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:45:59 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:47:41 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:55:20 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:55:57 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 17:57:30 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:01:25 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:02:03 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:02:44 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:06:18 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:07:00 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:08:44 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:11:48 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:13:34 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:15:17 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:24:37 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:25:08 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:26:35 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:28:07 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:28:44 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:29:19 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:30:02 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:31:52 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:33:45 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:34:23 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:35:01 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:35:33 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:37:36 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:38:02 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 18:38:30 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 19:24:51 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 19:34:53 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 19:37:06 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 19:38:23 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 19:40:03 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 19:43:06 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 19:47:26 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 19:50:36 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 19:53:29 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 19:54:37 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 20:03:44 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 20:07:21 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 20:08:28 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 20:10:19 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 20:13:44 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 20:15:15 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 20:27:58 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 20:29:20 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 20:32:17 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 20:34:06 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 20:36:30 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 20:38:23 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 20:46:35 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 20:48:34 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 20:58:17 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 21:30:44 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 21:33:29 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 21:35:08 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 21:39:35 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 21:52:07 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 21:54:00 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 21:55:20 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 22:09:04 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 22:10:42 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 22:39:24 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 22:40:54 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 22:42:26 IST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 22:45:02 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 00:33:49 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 19:40:45 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 19:46:52 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 19:48:08 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:17:38 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:18:31 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:21:01 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:21:26 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:21:46 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:22:33 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:22:56 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:23:19 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:28:24 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:28:57 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:29:31 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:30:55 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:31:31 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:32:08 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:33:15 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:33:52 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:34:41 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:37:47 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:38:15 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:38:44 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:39:53 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:40:30 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:41:09 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:52:08 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:54:05 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:56:01 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 21:58:43 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:00:33 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:01:14 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:09:33 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:10:09 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:11:50 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:13:21 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:15:04 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:16:52 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:19:28 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:21:29 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:23:12 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:25:13 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:27:03 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:27:38 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:29:13 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:31:14 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:31:47 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:34:36 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:35:05 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:36:41 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:37:06 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:37:32 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:38:25 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:38:48 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:39:12 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:44:53 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:46:32 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:48:38 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:52:32 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:53:08 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:54:52 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:59:13 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 22:59:52 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:01:43 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:07:10 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:08:44 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:09:14 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:11:16 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:13:00 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:13:30 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:14:34 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:15:08 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:15:55 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:19:28 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:20:10 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:21:54 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:27:32 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:29:13 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:30:45 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:32:17 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:34:38 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:35:12 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:37:48 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:38:15 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:41:05 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:42:40 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:44:22 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:44:53 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:46:21 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:48:58 IST 2025</t>
+  </si>
+  <si>
+    <t>Tue Dec 16 23:50:33 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:01:01 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:01:37 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:03:09 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:03:29 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:03:52 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:04:47 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:05:08 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:05:29 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:11:30 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:12:00 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:12:31 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:13:36 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:15:21 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:17:04 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:18:10 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:19:56 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:21:40 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:26:12 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:28:20 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:29:53 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:31:04 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:32:48 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:33:23 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:35:52 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:36:36 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:38:27 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:40:54 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:42:44 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:43:23 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:54:26 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:56:14 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:57:56 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 02:58:28 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:00:09 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:00:51 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:02:36 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:04:42 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:06:15 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:08:09 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:10:04 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:12:47 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:13:20 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:15:21 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:15:54 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:16:44 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:17:06 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:18:38 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:18:59 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:19:23 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:20:14 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:20:36 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:21:01 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:26:07 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:26:43 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:28:17 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:32:06 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:33:49 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:36:28 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:38:39 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:39:11 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:41:54 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:49:35 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:51:07 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:51:34 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:52:34 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:54:13 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:55:50 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:59:14 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 03:59:49 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:01:50 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:04:42 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:05:18 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:05:53 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:14:09 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:14:45 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:16:25 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:17:58 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:19:26 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:20:00 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:22:22 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:23:46 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:25:26 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:26:57 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:28:42 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:30:27 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:32:00 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:32:31 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 04:34:32 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 12:41:30 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 12:42:14 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 12:44:06 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 12:44:38 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 12:45:00 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 12:45:42 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 12:46:11 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 12:46:34 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 12:51:33 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 12:53:16 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 12:54:59 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 12:58:27 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 12:59:03 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 12:59:40 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 13:02:02 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 13:02:40 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 13:04:30 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 13:06:45 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 13:08:17 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 13:09:56 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 13:13:20 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 13:13:57 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 13:16:08 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 13:20:08 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 19:49:14 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 19:49:35 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 19:51:25 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 19:51:51 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 19:52:10 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 19:52:48 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 19:53:07 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 19:53:36 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 19:58:57 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 20:00:32 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 20:01:02 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 20:02:55 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 20:03:24 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 20:03:53 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 20:06:03 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 20:07:43 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 20:10:19 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 20:12:23 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 20:12:53 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 17 20:14:29 IST 2025</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -386,21 +1686,21 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
+    <xf applyAlignment="1" applyBorder="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="0" numFmtId="49" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf applyBorder="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="0" numFmtId="49" xfId="0"/>
+    <xf applyBorder="1" borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle builtinId="0" name="Normal" xfId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -417,10 +1717,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -455,7 +1755,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin panose="020F0302020204030204" typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -490,7 +1790,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin panose="020F0502020204030204" typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -584,21 +1884,21 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cap="flat" cmpd="sng" w="6350">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cap="flat" cmpd="sng" w="12700">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cap="flat" cmpd="sng" w="19050">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -615,7 +1915,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw algn="ctr" blurRad="57150" dir="5400000" dist="19050" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -667,21 +1967,21 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" name="Office Theme" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="26" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" customWidth="true" width="26.0" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -727,10 +2027,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>71</v>
+        <v>463</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>23</v>
@@ -766,7 +2066,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
   <headerFooter>
     <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
   </headerFooter>
@@ -774,14 +2074,14 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B84B2224-A06F-477C-8FF6-AF4C244AA0CE}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B84B2224-A06F-477C-8FF6-AF4C244AA0CE}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -827,10 +2127,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>76</v>
+        <v>468</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -864,16 +2164,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C366B0B2-5D78-426C-AEBB-C29C53584E7F}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C366B0B2-5D78-426C-AEBB-C29C53584E7F}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -919,10 +2219,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>79</v>
+        <v>471</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -956,16 +2256,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35ACE39D-499D-49B4-BFD2-CDDE6D0F8728}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35ACE39D-499D-49B4-BFD2-CDDE6D0F8728}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1011,10 +2311,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>75</v>
+        <v>467</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1048,16 +2348,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29FACBAA-68A5-4A1D-8E32-A4AA8B032AE1}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29FACBAA-68A5-4A1D-8E32-A4AA8B032AE1}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1106,7 +2406,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>42</v>
+        <v>502</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1140,16 +2440,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{924F2B64-1D9A-415C-B98F-EB7A7BAB8DD9}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{924F2B64-1D9A-415C-B98F-EB7A7BAB8DD9}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1195,10 +2495,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>50</v>
+        <v>509</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1232,16 +2532,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A084124A-76B7-4B99-A6AD-5B2A169F9B8A}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A084124A-76B7-4B99-A6AD-5B2A169F9B8A}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1290,7 +2590,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>510</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1324,16 +2624,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0332CA16-31EB-4917-9936-860E79D3523B}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0332CA16-31EB-4917-9936-860E79D3523B}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1382,7 +2682,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>52</v>
+        <v>511</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1416,16 +2716,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF1E53DD-391D-45C7-A26E-A3CBEF12F623}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF1E53DD-391D-45C7-A26E-A3CBEF12F623}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1474,7 +2774,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>512</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1508,16 +2808,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65676D18-4455-410B-8CF0-024536C3D41C}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65676D18-4455-410B-8CF0-024536C3D41C}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1566,7 +2866,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>513</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1600,16 +2900,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06203600-C68B-4759-93E3-003ACDDD00D9}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06203600-C68B-4759-93E3-003ACDDD00D9}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1655,10 +2955,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>55</v>
+        <v>514</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1692,16 +2992,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{188BD99A-2280-478C-8415-3AF3B8D2E566}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{188BD99A-2280-478C-8415-3AF3B8D2E566}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1747,10 +3047,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>72</v>
+        <v>464</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>23</v>
@@ -1786,16 +3086,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{044EB785-1D8B-4520-A589-98FB5248CE3B}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{044EB785-1D8B-4520-A589-98FB5248CE3B}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1841,10 +3141,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>515</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1878,16 +3178,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAB2259B-110A-4E54-AAE6-DB14B9EB5171}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAB2259B-110A-4E54-AAE6-DB14B9EB5171}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1933,10 +3233,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>516</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1970,16 +3270,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE735932-BE48-4F0B-B6E0-1AACE863DBE6}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE735932-BE48-4F0B-B6E0-1AACE863DBE6}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2025,10 +3325,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>58</v>
+        <v>517</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2062,16 +3362,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4FDA41C-A48E-4DF7-9F3C-4EA15B85EA24}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4FDA41C-A48E-4DF7-9F3C-4EA15B85EA24}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2120,7 +3420,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>61</v>
+        <v>497</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2154,16 +3454,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6653DFE2-5232-47EC-B0F1-E3DFB6BF3E7A}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6653DFE2-5232-47EC-B0F1-E3DFB6BF3E7A}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2209,10 +3509,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>499</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2246,16 +3546,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C026E37F-098F-42E5-92AB-1E317624CC4D}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C026E37F-098F-42E5-92AB-1E317624CC4D}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2301,10 +3601,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>498</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2338,19 +3638,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDE16B14-240B-4522-A71A-377E72FADE1F}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDE16B14-240B-4522-A71A-377E72FADE1F}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="26" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" customWidth="true" width="26.0" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2427,19 +3727,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37E5825C-6EEF-49AA-9880-B92945E2442C}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37E5825C-6EEF-49AA-9880-B92945E2442C}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2516,19 +3816,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63B10A84-4465-4F3C-AB05-F2529380B3EA}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63B10A84-4465-4F3C-AB05-F2529380B3EA}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="26" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" customWidth="true" width="26.0" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2607,19 +3907,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD262109-C636-4152-9E03-BF0F49D8C917}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD262109-C636-4152-9E03-BF0F49D8C917}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="26" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" customWidth="true" width="26.0" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2704,16 +4004,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56CB3A07-E958-4D14-B792-C4C5D72CD8EA}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56CB3A07-E958-4D14-B792-C4C5D72CD8EA}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2759,10 +4059,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>501</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2796,19 +4096,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FBEB25C-002A-46ED-B528-BBFB127AD6B5}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FBEB25C-002A-46ED-B528-BBFB127AD6B5}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2891,19 +4191,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78A3C05C-8E29-42C3-A89E-8ED671B7BB31}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78A3C05C-8E29-42C3-A89E-8ED671B7BB31}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2986,16 +4286,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDB610E4-D8A9-4F86-99AA-691BCAA68B9C}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDB610E4-D8A9-4F86-99AA-691BCAA68B9C}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3041,10 +4341,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>500</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3078,16 +4378,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D3C025A-C3F4-4ABF-9C60-AA1DCCB0BC50}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D3C025A-C3F4-4ABF-9C60-AA1DCCB0BC50}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3133,10 +4433,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>457</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3170,16 +4470,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A067396-2824-448F-9289-4B8D3E2041FE}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A067396-2824-448F-9289-4B8D3E2041FE}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3225,10 +4525,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>66</v>
+        <v>458</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3262,16 +4562,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AECE1F9-32F0-48E5-B835-168A7EF42FA8}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AECE1F9-32F0-48E5-B835-168A7EF42FA8}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3320,7 +4620,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>459</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3354,16 +4654,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AEB8BAF-D441-4510-B01C-E6A2F0E35EEA}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AEB8BAF-D441-4510-B01C-E6A2F0E35EEA}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3412,7 +4712,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>68</v>
+        <v>460</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3446,16 +4746,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4CCB5A6-D07A-4BC3-BD3B-767113A862D2}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4CCB5A6-D07A-4BC3-BD3B-767113A862D2}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3504,7 +4804,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>461</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3538,19 +4838,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55F93338-8AAA-4B19-8B9D-4771302FEFC0}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55F93338-8AAA-4B19-8B9D-4771302FEFC0}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="17.21875" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" customWidth="true" width="17.21875" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3596,10 +4896,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>470</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>25</v>
@@ -3635,19 +4935,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EC6E653-D4E4-4FCF-8BD0-11D4CBABA3A9}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EC6E653-D4E4-4FCF-8BD0-11D4CBABA3A9}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3696,7 +4996,7 @@
         <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>77</v>
+        <v>469</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -3730,16 +5030,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{893E9D9E-A65A-420C-985F-4AFBCEBD5458}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{893E9D9E-A65A-420C-985F-4AFBCEBD5458}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3788,7 +5088,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>70</v>
+        <v>462</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3822,19 +5122,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF98BAE0-3DBA-4724-A623-84E06EAD3F5D}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF98BAE0-3DBA-4724-A623-84E06EAD3F5D}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3880,10 +5180,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>519</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -3917,16 +5217,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36CD5E31-F635-4FC0-9668-1419F01D6942}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36CD5E31-F635-4FC0-9668-1419F01D6942}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3975,7 +5275,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>47</v>
+        <v>507</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4009,19 +5309,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBD2F0AE-7828-442C-A2B3-21D0EBE7331D}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBD2F0AE-7828-442C-A2B3-21D0EBE7331D}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4070,7 +5370,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>504</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4104,16 +5404,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62E2C147-58C7-49F8-940A-3E37DE049451}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62E2C147-58C7-49F8-940A-3E37DE049451}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4159,10 +5459,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>81</v>
+        <v>473</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4196,16 +5496,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DC79200-E4B3-4160-86F6-78B06F6EA2C0}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DC79200-E4B3-4160-86F6-78B06F6EA2C0}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4254,7 +5554,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>84</v>
+        <v>476</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4288,16 +5588,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{026E9C75-7C58-441D-91D6-25552A135B0A}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{026E9C75-7C58-441D-91D6-25552A135B0A}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4343,10 +5643,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>80</v>
+        <v>472</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4380,16 +5680,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D307F9B9-84A6-4F70-AF5F-E09C0B70177D}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D307F9B9-84A6-4F70-AF5F-E09C0B70177D}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4438,7 +5738,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>82</v>
+        <v>474</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4472,16 +5772,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CED210A-15BA-4154-A75C-369A0BF113DA}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CED210A-15BA-4154-A75C-369A0BF113DA}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4527,10 +5827,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>83</v>
+        <v>475</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>26</v>
@@ -4566,16 +5866,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13CCEC20-911A-47BC-B790-0438DD3BE26D}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13CCEC20-911A-47BC-B790-0438DD3BE26D}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4621,10 +5921,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>60</v>
+        <v>520</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4658,16 +5958,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEE927C8-204D-43C3-9530-F9F77785B40B}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEE927C8-204D-43C3-9530-F9F77785B40B}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4716,7 +6016,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>45</v>
+        <v>505</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4750,16 +6050,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F88BD42D-CC7A-48FA-8796-B59D2B587379}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F88BD42D-CC7A-48FA-8796-B59D2B587379}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4808,7 +6108,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>74</v>
+        <v>466</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4842,16 +6142,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAABB2E9-54E4-4860-85B4-28F35D889E47}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAABB2E9-54E4-4860-85B4-28F35D889E47}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4900,7 +6200,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>508</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4934,19 +6234,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B65B44A-04F0-4B2C-962C-6C956F0737B9}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B65B44A-04F0-4B2C-962C-6C956F0737B9}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="26" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" customWidth="true" width="26.0" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4995,7 +6295,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>503</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -5029,16 +6329,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A462096B-4AF9-4B81-B6B6-00EE8E7EF270}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A462096B-4AF9-4B81-B6B6-00EE8E7EF270}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5087,7 +6387,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>46</v>
+        <v>506</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -5121,19 +6421,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04E9BD2B-9C3A-4D4A-991E-C6044AE36784}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04E9BD2B-9C3A-4D4A-991E-C6044AE36784}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="26" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" customWidth="true" width="26.0" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5182,7 +6482,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>518</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -5216,19 +6516,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A723C119-E528-48BF-99DE-522307C92146}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A723C119-E528-48BF-99DE-522307C92146}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="19" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" customWidth="true" width="19.0" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5274,10 +6574,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>73</v>
+        <v>465</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>
@@ -5313,6 +6613,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fixes for IWP-27 bootstrap
</commit_message>
<xml_diff>
--- a/KatalonData/BWPBootstrapData/BWPACHData.xlsx
+++ b/KatalonData/BWPBootstrapData/BWPACHData.xlsx
@@ -1,72 +1,72 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t476046\Documents\VPS-Katalon-feature-VRelay\KatalonData\BWPBootstrapData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55E1A0A7-BC18-4D8D-8BEC-EB12C7564819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr documentId="13_ncr:1_{55E1A0A7-BC18-4D8D-8BEC-EB12C7564819}" revIDLastSave="0" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="27" activeTab="30" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="30" firstSheet="27" windowHeight="12456" windowWidth="23256" xWindow="-108" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" yWindow="-108"/>
   </bookViews>
   <sheets>
-    <sheet name="PayNowCorpNoCF" sheetId="1" r:id="rId1"/>
-    <sheet name="PayNowCorpNoCFOnly" sheetId="13" r:id="rId2"/>
-    <sheet name="ACMismatchCorp" sheetId="25" r:id="rId3"/>
-    <sheet name="PayNowCorpDCF" sheetId="8" r:id="rId4"/>
-    <sheet name="PayNowCorpSCF" sheetId="7" r:id="rId5"/>
-    <sheet name="MaxAmountErrorCorp" sheetId="19" r:id="rId6"/>
-    <sheet name="MinAmountErrorCorp" sheetId="22" r:id="rId7"/>
-    <sheet name="NoModifyAmountCorp" sheetId="16" r:id="rId8"/>
-    <sheet name="PayNowCorpNoCFReqFields" sheetId="2" r:id="rId9"/>
-    <sheet name="PayNowPCNoCF" sheetId="3" r:id="rId10"/>
-    <sheet name="PayNowPCSCF" sheetId="9" r:id="rId11"/>
-    <sheet name="PayNowPCDCF" sheetId="11" r:id="rId12"/>
-    <sheet name="ACMismatchPC" sheetId="26" r:id="rId13"/>
-    <sheet name="DualCFCeilingCorp" sheetId="27" r:id="rId14"/>
-    <sheet name="DualCFCeilingPC" sheetId="28" r:id="rId15"/>
-    <sheet name="DualCFCeilingPS" sheetId="29" r:id="rId16"/>
-    <sheet name="DualCFFlatCorp" sheetId="30" r:id="rId17"/>
-    <sheet name="DualCFFlatPC" sheetId="31" r:id="rId18"/>
-    <sheet name="DualCFFlatPS" sheetId="32" r:id="rId19"/>
-    <sheet name="DualCFPercentageCorp" sheetId="33" r:id="rId20"/>
-    <sheet name="DualCFPercentagePC" sheetId="34" r:id="rId21"/>
-    <sheet name="DualCFPercentagePS" sheetId="35" r:id="rId22"/>
-    <sheet name="SingleCFCeilingCorp" sheetId="36" r:id="rId23"/>
-    <sheet name="SingleCFCeilingPS" sheetId="38" r:id="rId24"/>
-    <sheet name="SingleCFCeilingPC" sheetId="37" r:id="rId25"/>
-    <sheet name="MissingReqFieldsCorp" sheetId="45" r:id="rId26"/>
-    <sheet name="MissingReqFieldsPersonalACH" sheetId="46" r:id="rId27"/>
-    <sheet name="ModifyPaymentsCorp1" sheetId="47" r:id="rId28"/>
-    <sheet name="ModifyPaymentsCorp2" sheetId="48" r:id="rId29"/>
-    <sheet name="ModifyPaymentsPC1" sheetId="49" r:id="rId30"/>
-    <sheet name="ModifyPaymentsPC2" sheetId="50" r:id="rId31"/>
-    <sheet name="SingleCFFlatCorp" sheetId="39" r:id="rId32"/>
-    <sheet name="SingleCFFlatPC" sheetId="40" r:id="rId33"/>
-    <sheet name="SingleCFFlatPS" sheetId="41" r:id="rId34"/>
-    <sheet name="SingleCFPercentageCorp" sheetId="42" r:id="rId35"/>
-    <sheet name="SingleCFPercentagePC" sheetId="43" r:id="rId36"/>
-    <sheet name="SingleCFPercentagePS" sheetId="44" r:id="rId37"/>
-    <sheet name="PayNowPCNoCFReqFields" sheetId="4" r:id="rId38"/>
-    <sheet name="PayNowPCNoCFOnly" sheetId="14" r:id="rId39"/>
-    <sheet name="NoModifyAmountPC" sheetId="17" r:id="rId40"/>
-    <sheet name="MinAmountErrorPC" sheetId="23" r:id="rId41"/>
-    <sheet name="MaxAmountErrorPC" sheetId="20" r:id="rId42"/>
-    <sheet name="PayNowPSNoCF" sheetId="5" r:id="rId43"/>
-    <sheet name="PayNowPSSCF" sheetId="10" r:id="rId44"/>
-    <sheet name="PayNowPSDCF" sheetId="12" r:id="rId45"/>
-    <sheet name="PayNowPSNoCFOnly" sheetId="15" r:id="rId46"/>
-    <sheet name="PayNowPSNoCFReqFields" sheetId="6" r:id="rId47"/>
-    <sheet name="NoModifyAmountPS" sheetId="18" r:id="rId48"/>
-    <sheet name="MaxAmountErrorPS" sheetId="21" r:id="rId49"/>
-    <sheet name="MinAmountErrorPS" sheetId="24" r:id="rId50"/>
+    <sheet name="PayNowCorpNoCF" r:id="rId1" sheetId="1"/>
+    <sheet name="PayNowCorpNoCFOnly" r:id="rId2" sheetId="13"/>
+    <sheet name="ACMismatchCorp" r:id="rId3" sheetId="25"/>
+    <sheet name="PayNowCorpDCF" r:id="rId4" sheetId="8"/>
+    <sheet name="PayNowCorpSCF" r:id="rId5" sheetId="7"/>
+    <sheet name="MaxAmountErrorCorp" r:id="rId6" sheetId="19"/>
+    <sheet name="MinAmountErrorCorp" r:id="rId7" sheetId="22"/>
+    <sheet name="NoModifyAmountCorp" r:id="rId8" sheetId="16"/>
+    <sheet name="PayNowCorpNoCFReqFields" r:id="rId9" sheetId="2"/>
+    <sheet name="PayNowPCNoCF" r:id="rId10" sheetId="3"/>
+    <sheet name="PayNowPCSCF" r:id="rId11" sheetId="9"/>
+    <sheet name="PayNowPCDCF" r:id="rId12" sheetId="11"/>
+    <sheet name="ACMismatchPC" r:id="rId13" sheetId="26"/>
+    <sheet name="DualCFCeilingCorp" r:id="rId14" sheetId="27"/>
+    <sheet name="DualCFCeilingPC" r:id="rId15" sheetId="28"/>
+    <sheet name="DualCFCeilingPS" r:id="rId16" sheetId="29"/>
+    <sheet name="DualCFFlatCorp" r:id="rId17" sheetId="30"/>
+    <sheet name="DualCFFlatPC" r:id="rId18" sheetId="31"/>
+    <sheet name="DualCFFlatPS" r:id="rId19" sheetId="32"/>
+    <sheet name="DualCFPercentageCorp" r:id="rId20" sheetId="33"/>
+    <sheet name="DualCFPercentagePC" r:id="rId21" sheetId="34"/>
+    <sheet name="DualCFPercentagePS" r:id="rId22" sheetId="35"/>
+    <sheet name="SingleCFCeilingCorp" r:id="rId23" sheetId="36"/>
+    <sheet name="SingleCFCeilingPS" r:id="rId24" sheetId="38"/>
+    <sheet name="SingleCFCeilingPC" r:id="rId25" sheetId="37"/>
+    <sheet name="MissingReqFieldsCorp" r:id="rId26" sheetId="45"/>
+    <sheet name="MissingReqFieldsPersonalACH" r:id="rId27" sheetId="46"/>
+    <sheet name="ModifyPaymentsCorp1" r:id="rId28" sheetId="47"/>
+    <sheet name="ModifyPaymentsCorp2" r:id="rId29" sheetId="48"/>
+    <sheet name="ModifyPaymentsPC1" r:id="rId30" sheetId="49"/>
+    <sheet name="ModifyPaymentsPC2" r:id="rId31" sheetId="50"/>
+    <sheet name="SingleCFFlatCorp" r:id="rId32" sheetId="39"/>
+    <sheet name="SingleCFFlatPC" r:id="rId33" sheetId="40"/>
+    <sheet name="SingleCFFlatPS" r:id="rId34" sheetId="41"/>
+    <sheet name="SingleCFPercentageCorp" r:id="rId35" sheetId="42"/>
+    <sheet name="SingleCFPercentagePC" r:id="rId36" sheetId="43"/>
+    <sheet name="SingleCFPercentagePS" r:id="rId37" sheetId="44"/>
+    <sheet name="PayNowPCNoCFReqFields" r:id="rId38" sheetId="4"/>
+    <sheet name="PayNowPCNoCFOnly" r:id="rId39" sheetId="14"/>
+    <sheet name="NoModifyAmountPC" r:id="rId40" sheetId="17"/>
+    <sheet name="MinAmountErrorPC" r:id="rId41" sheetId="23"/>
+    <sheet name="MaxAmountErrorPC" r:id="rId42" sheetId="20"/>
+    <sheet name="PayNowPSNoCF" r:id="rId43" sheetId="5"/>
+    <sheet name="PayNowPSSCF" r:id="rId44" sheetId="10"/>
+    <sheet name="PayNowPSDCF" r:id="rId45" sheetId="12"/>
+    <sheet name="PayNowPSNoCFOnly" r:id="rId46" sheetId="15"/>
+    <sheet name="PayNowPSNoCFReqFields" r:id="rId47" sheetId="6"/>
+    <sheet name="NoModifyAmountPS" r:id="rId48" sheetId="18"/>
+    <sheet name="MaxAmountErrorPS" r:id="rId49" sheetId="21"/>
+    <sheet name="MinAmountErrorPS" r:id="rId50" sheetId="24"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1251" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2199" uniqueCount="326">
   <si>
     <t>Result</t>
   </si>
@@ -338,12 +338,727 @@
   </si>
   <si>
     <t>8</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Fri Jan 16 19:41:15 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 19:42:03 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 19:46:35 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 19:46:59 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 19:47:21 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 19:48:11 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 19:48:39 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 19:49:01 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 19:59:00 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 19:59:32 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:00:06 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:01:13 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:01:55 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:02:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:03:55 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:04:35 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:05:10 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:07:50 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:08:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:08:55 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:10:07 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:10:42 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:12:50 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:13:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:15:38 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:17:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:18:05 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:18:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:20:14 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:20:57 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:21:38 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:29:50 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:30:28 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:31:56 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:33:27 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:34:03 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:34:39 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:35:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:36:06 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:36:42 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:37:16 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:38:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:40:22 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:41:54 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:43:25 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:45:02 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:45:44 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:48:44 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:49:25 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:50:05 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:51:42 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:53:55 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:54:31 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:56:06 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:58:17 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 20:58:53 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:01:03 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:03:12 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:04:51 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:05:22 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:06:17 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:06:50 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:10:32 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:10:52 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:11:10 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:11:27 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:12:05 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:12:28 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:12:54 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:20:52 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:21:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:21:50 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:24:30 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:25:05 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:25:35 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:26:05 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:28:46 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:29:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:30:25 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:30:56 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:46:12 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:47:40 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:49:11 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:49:39 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:51:10 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:52:44 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:53:13 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:58:03 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:58:34 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 21:59:05 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:01:12 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:02:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:02:54 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:03:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:04:43 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:05:21 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:05:57 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:11:56 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:12:25 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:13:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:14:16 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:17:05 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:18:51 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:19:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:19:44 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:20:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:20:52 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:22:48 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:24:12 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:24:40 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:26:03 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:28:00 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:28:27 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:29:02 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:29:38 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:30:05 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:31:30 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:32:00 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:32:34 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:34:05 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:35:30 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:36:54 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jan 16 22:38:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:34:07 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:34:47 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:39:22 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:39:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:40:13 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:41:00 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:41:25 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:41:52 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:42:15 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:42:40 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:49:36 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:50:07 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:50:40 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:52:45 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:53:51 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:54:29 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:55:07 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:57:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:58:25 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 00:59:01 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:00:16 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:01:45 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:03:14 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:04:43 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:05:16 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:05:47 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:06:58 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:07:35 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:09:43 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:10:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:11:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:12:19 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:13:01 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:14:24 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:15:05 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:17:47 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:18:33 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:21:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:27:41 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:28:15 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:28:45 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:29:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:29:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:30:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:30:59 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:32:59 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:33:30 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:35:00 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:35:29 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:35:58 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:36:35 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:37:08 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:37:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:39:34 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:41:36 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:43:02 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:44:31 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:46:02 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:47:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:48:08 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:48:50 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:49:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:49:39 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:52:10 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:52:25 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:52:41 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:53:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:53:34 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 01:53:50 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:03:10 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:03:40 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:05:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:06:03 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:09:31 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:09:57 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:10:30 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:12:55 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:13:23 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:15:55 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:16:21 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:32:06 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:33:28 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:33:52 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:34:15 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:37:05 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:37:34 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:38:08 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:39:23 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:39:55 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:40:31 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:41:41 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:42:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:42:56 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:55:55 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:56:25 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:57:51 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:58:19 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 02:58:51 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 03:00:29 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 03:00:59 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 03:01:28 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 03:01:56 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 03:02:27 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 03:03:50 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 03:05:38 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 03:06:10 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 03:06:43 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 03:07:11 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 03:07:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 03:08:02 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 03:08:29 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 17 03:11:09 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Jan 19 19:36:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Jan 19 19:39:20 IST 2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -386,21 +1101,21 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
+    <xf applyAlignment="1" applyBorder="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="0" numFmtId="49" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf applyBorder="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="0" numFmtId="49" xfId="0"/>
+    <xf applyBorder="1" borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle builtinId="0" name="Normal" xfId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -417,10 +1132,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -455,7 +1170,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin panose="020F0302020204030204" typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -490,7 +1205,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin panose="020F0502020204030204" typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -584,21 +1299,21 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cap="flat" cmpd="sng" w="6350">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cap="flat" cmpd="sng" w="12700">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cap="flat" cmpd="sng" w="19050">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -615,7 +1330,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw algn="ctr" blurRad="57150" dir="5400000" dist="19050" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -667,21 +1382,21 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" name="Office Theme" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="26" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" customWidth="true" width="26.0" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -730,7 +1445,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>71</v>
+        <v>307</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>23</v>
@@ -766,7 +1481,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
   <headerFooter>
     <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
   </headerFooter>
@@ -774,14 +1489,14 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B84B2224-A06F-477C-8FF6-AF4C244AA0CE}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B84B2224-A06F-477C-8FF6-AF4C244AA0CE}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -830,7 +1545,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>76</v>
+        <v>312</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -864,16 +1579,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C366B0B2-5D78-426C-AEBB-C29C53584E7F}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C366B0B2-5D78-426C-AEBB-C29C53584E7F}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -922,7 +1637,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>79</v>
+        <v>317</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -956,16 +1671,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35ACE39D-499D-49B4-BFD2-CDDE6D0F8728}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35ACE39D-499D-49B4-BFD2-CDDE6D0F8728}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1014,7 +1729,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>75</v>
+        <v>311</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1048,16 +1763,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29FACBAA-68A5-4A1D-8E32-A4AA8B032AE1}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29FACBAA-68A5-4A1D-8E32-A4AA8B032AE1}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1106,7 +1821,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>42</v>
+        <v>274</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1140,16 +1855,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{924F2B64-1D9A-415C-B98F-EB7A7BAB8DD9}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{924F2B64-1D9A-415C-B98F-EB7A7BAB8DD9}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1198,7 +1913,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>50</v>
+        <v>281</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1232,16 +1947,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A084124A-76B7-4B99-A6AD-5B2A169F9B8A}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A084124A-76B7-4B99-A6AD-5B2A169F9B8A}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1290,7 +2005,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>283</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1324,16 +2039,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0332CA16-31EB-4917-9936-860E79D3523B}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0332CA16-31EB-4917-9936-860E79D3523B}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1382,7 +2097,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>52</v>
+        <v>284</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1416,16 +2131,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF1E53DD-391D-45C7-A26E-A3CBEF12F623}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF1E53DD-391D-45C7-A26E-A3CBEF12F623}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1474,7 +2189,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>285</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1508,16 +2223,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65676D18-4455-410B-8CF0-024536C3D41C}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65676D18-4455-410B-8CF0-024536C3D41C}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1566,7 +2281,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>286</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1600,16 +2315,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06203600-C68B-4759-93E3-003ACDDD00D9}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06203600-C68B-4759-93E3-003ACDDD00D9}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1658,7 +2373,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>55</v>
+        <v>287</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1692,16 +2407,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{188BD99A-2280-478C-8415-3AF3B8D2E566}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{188BD99A-2280-478C-8415-3AF3B8D2E566}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1750,7 +2465,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>72</v>
+        <v>308</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>23</v>
@@ -1786,16 +2501,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{044EB785-1D8B-4520-A589-98FB5248CE3B}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{044EB785-1D8B-4520-A589-98FB5248CE3B}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1844,7 +2559,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>288</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1878,16 +2593,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAB2259B-110A-4E54-AAE6-DB14B9EB5171}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAB2259B-110A-4E54-AAE6-DB14B9EB5171}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1936,7 +2651,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>290</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1970,16 +2685,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE735932-BE48-4F0B-B6E0-1AACE863DBE6}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE735932-BE48-4F0B-B6E0-1AACE863DBE6}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2025,10 +2740,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>58</v>
+        <v>291</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2062,16 +2777,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4FDA41C-A48E-4DF7-9F3C-4EA15B85EA24}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4FDA41C-A48E-4DF7-9F3C-4EA15B85EA24}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2120,7 +2835,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>61</v>
+        <v>296</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2154,16 +2869,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6653DFE2-5232-47EC-B0F1-E3DFB6BF3E7A}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6653DFE2-5232-47EC-B0F1-E3DFB6BF3E7A}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2212,7 +2927,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>298</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2246,16 +2961,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C026E37F-098F-42E5-92AB-1E317624CC4D}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C026E37F-098F-42E5-92AB-1E317624CC4D}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2304,7 +3019,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>297</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2338,19 +3053,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDE16B14-240B-4522-A71A-377E72FADE1F}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDE16B14-240B-4522-A71A-377E72FADE1F}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="26" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" customWidth="true" width="26.0" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2427,19 +3142,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37E5825C-6EEF-49AA-9880-B92945E2442C}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37E5825C-6EEF-49AA-9880-B92945E2442C}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2516,19 +3231,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63B10A84-4465-4F3C-AB05-F2529380B3EA}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63B10A84-4465-4F3C-AB05-F2529380B3EA}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="26" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" customWidth="true" width="26.0" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2607,19 +3322,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD262109-C636-4152-9E03-BF0F49D8C917}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD262109-C636-4152-9E03-BF0F49D8C917}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="26" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" customWidth="true" width="26.0" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2704,16 +3419,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56CB3A07-E958-4D14-B792-C4C5D72CD8EA}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56CB3A07-E958-4D14-B792-C4C5D72CD8EA}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2762,7 +3477,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>272</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2796,19 +3511,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FBEB25C-002A-46ED-B528-BBFB127AD6B5}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FBEB25C-002A-46ED-B528-BBFB127AD6B5}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2891,19 +3606,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78A3C05C-8E29-42C3-A89E-8ED671B7BB31}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78A3C05C-8E29-42C3-A89E-8ED671B7BB31}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2986,16 +3701,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDB610E4-D8A9-4F86-99AA-691BCAA68B9C}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDB610E4-D8A9-4F86-99AA-691BCAA68B9C}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3044,7 +3759,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>299</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3078,16 +3793,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D3C025A-C3F4-4ABF-9C60-AA1DCCB0BC50}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D3C025A-C3F4-4ABF-9C60-AA1DCCB0BC50}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3136,7 +3851,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>300</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3170,16 +3885,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A067396-2824-448F-9289-4B8D3E2041FE}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A067396-2824-448F-9289-4B8D3E2041FE}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3228,7 +3943,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>66</v>
+        <v>301</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3262,16 +3977,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AECE1F9-32F0-48E5-B835-168A7EF42FA8}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AECE1F9-32F0-48E5-B835-168A7EF42FA8}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3320,7 +4035,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>302</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3354,16 +4069,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AEB8BAF-D441-4510-B01C-E6A2F0E35EEA}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AEB8BAF-D441-4510-B01C-E6A2F0E35EEA}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3412,7 +4127,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>68</v>
+        <v>303</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3446,16 +4161,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4CCB5A6-D07A-4BC3-BD3B-767113A862D2}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4CCB5A6-D07A-4BC3-BD3B-767113A862D2}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3504,7 +4219,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>304</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3538,19 +4253,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55F93338-8AAA-4B19-8B9D-4771302FEFC0}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55F93338-8AAA-4B19-8B9D-4771302FEFC0}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="17.21875" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" customWidth="true" width="17.21875" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3599,7 +4314,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>316</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>25</v>
@@ -3635,19 +4350,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EC6E653-D4E4-4FCF-8BD0-11D4CBABA3A9}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EC6E653-D4E4-4FCF-8BD0-11D4CBABA3A9}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3693,10 +4408,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>77</v>
+        <v>313</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -3730,16 +4445,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{893E9D9E-A65A-420C-985F-4AFBCEBD5458}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{893E9D9E-A65A-420C-985F-4AFBCEBD5458}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3788,7 +4503,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>70</v>
+        <v>305</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3822,19 +4537,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF98BAE0-3DBA-4724-A623-84E06EAD3F5D}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF98BAE0-3DBA-4724-A623-84E06EAD3F5D}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3883,7 +4598,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>294</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -3917,16 +4632,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36CD5E31-F635-4FC0-9668-1419F01D6942}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36CD5E31-F635-4FC0-9668-1419F01D6942}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3975,7 +4690,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>47</v>
+        <v>279</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4009,19 +4724,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBD2F0AE-7828-442C-A2B3-21D0EBE7331D}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBD2F0AE-7828-442C-A2B3-21D0EBE7331D}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="8.44140625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4070,7 +4785,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>276</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4104,16 +4819,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62E2C147-58C7-49F8-940A-3E37DE049451}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62E2C147-58C7-49F8-940A-3E37DE049451}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4162,7 +4877,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>81</v>
+        <v>319</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4196,16 +4911,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DC79200-E4B3-4160-86F6-78B06F6EA2C0}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DC79200-E4B3-4160-86F6-78B06F6EA2C0}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4254,7 +4969,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>84</v>
+        <v>323</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4288,16 +5003,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{026E9C75-7C58-441D-91D6-25552A135B0A}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{026E9C75-7C58-441D-91D6-25552A135B0A}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4346,7 +5061,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>80</v>
+        <v>318</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4380,16 +5095,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D307F9B9-84A6-4F70-AF5F-E09C0B70177D}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D307F9B9-84A6-4F70-AF5F-E09C0B70177D}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4438,7 +5153,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>82</v>
+        <v>325</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4472,16 +5187,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CED210A-15BA-4154-A75C-369A0BF113DA}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CED210A-15BA-4154-A75C-369A0BF113DA}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4530,7 +5245,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>83</v>
+        <v>321</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>26</v>
@@ -4566,16 +5281,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13CCEC20-911A-47BC-B790-0438DD3BE26D}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13CCEC20-911A-47BC-B790-0438DD3BE26D}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4624,7 +5339,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>60</v>
+        <v>295</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4658,16 +5373,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEE927C8-204D-43C3-9530-F9F77785B40B}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEE927C8-204D-43C3-9530-F9F77785B40B}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4716,7 +5431,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>45</v>
+        <v>277</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4750,16 +5465,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F88BD42D-CC7A-48FA-8796-B59D2B587379}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F88BD42D-CC7A-48FA-8796-B59D2B587379}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4808,7 +5523,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>74</v>
+        <v>310</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4842,16 +5557,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAABB2E9-54E4-4860-85B4-28F35D889E47}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAABB2E9-54E4-4860-85B4-28F35D889E47}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4900,7 +5615,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>280</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4934,19 +5649,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B65B44A-04F0-4B2C-962C-6C956F0737B9}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B65B44A-04F0-4B2C-962C-6C956F0737B9}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="26" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" customWidth="true" width="26.0" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4995,7 +5710,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>275</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -5029,16 +5744,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A462096B-4AF9-4B81-B6B6-00EE8E7EF270}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A462096B-4AF9-4B81-B6B6-00EE8E7EF270}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5087,7 +5802,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>46</v>
+        <v>278</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -5121,19 +5836,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04E9BD2B-9C3A-4D4A-991E-C6044AE36784}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04E9BD2B-9C3A-4D4A-991E-C6044AE36784}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="26" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" customWidth="true" width="26.0" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5182,7 +5897,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>293</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -5216,19 +5931,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A723C119-E528-48BF-99DE-522307C92146}">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A723C119-E528-48BF-99DE-522307C92146}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="19" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" customWidth="true" width="19.0" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5277,7 +5992,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>73</v>
+        <v>309</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>
@@ -5313,6 +6028,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
IWP 3.0 Bootstrap Regression Testcases added
</commit_message>
<xml_diff>
--- a/KatalonData/BWPBootstrapData/BWPACHData.xlsx
+++ b/KatalonData/BWPBootstrapData/BWPACHData.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2199" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2679" uniqueCount="446">
   <si>
     <t>Result</t>
   </si>
@@ -1052,6 +1052,366 @@
   </si>
   <si>
     <t>Mon Jan 19 19:39:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 21:55:56 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 21:56:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 21:58:19 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 21:58:41 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 21:59:06 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 21:59:47 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:00:07 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:00:32 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:05:46 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:06:17 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:06:51 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:07:54 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:08:33 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:09:15 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:10:27 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:11:01 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:11:36 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:15:52 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:17:25 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:19:01 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:20:33 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:21:03 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:21:39 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:22:46 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:23:27 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:24:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:25:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:26:01 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:26:41 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:28:00 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:28:42 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:29:21 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:37:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:37:38 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:39:09 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:39:54 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:41:22 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:42:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:44:19 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:44:50 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:46:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:46:55 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:47:35 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:48:10 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:48:47 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:50:15 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:51:48 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:53:17 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:53:53 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:54:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:55:08 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 22:57:44 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:00:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:02:57 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:05:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:07:14 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:09:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:11:46 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:12:23 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:13:51 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:14:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:14:59 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:15:38 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:16:01 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:17:32 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:17:54 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:18:23 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:18:48 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:19:36 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:20:01 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:20:22 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:27:43 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:28:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:28:51 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:29:58 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:30:43 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:31:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:32:42 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:33:23 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:34:03 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:36:41 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:39:23 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:47:48 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:48:17 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:49:42 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:50:09 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:51:14 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:51:50 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:52:25 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:53:35 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:54:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:57:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:58:02 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 06 23:59:27 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:00:07 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:00:48 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:11:34 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:13:16 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:13:46 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:15:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:15:50 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:16:23 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:17:00 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:17:43 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:18:13 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:20:43 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:22:11 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:22:57 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:24:24 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:26:03 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:26:43 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:29:32 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:30:24 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:30:59 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:33:57 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:36:25 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:37:12 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:40:44 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 00:41:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu May 07 21:00:28 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -1445,7 +1805,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>307</v>
+        <v>423</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>23</v>
@@ -1545,7 +1905,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>312</v>
+        <v>429</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -1637,7 +1997,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>317</v>
+        <v>437</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1729,7 +2089,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>311</v>
+        <v>428</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1821,7 +2181,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>274</v>
+        <v>389</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1913,7 +2273,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>281</v>
+        <v>397</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2005,7 +2365,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>283</v>
+        <v>398</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2097,7 +2457,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>284</v>
+        <v>399</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2189,7 +2549,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>285</v>
+        <v>400</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2281,7 +2641,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>286</v>
+        <v>401</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2373,7 +2733,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>287</v>
+        <v>402</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2465,7 +2825,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>308</v>
+        <v>425</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>23</v>
@@ -2559,7 +2919,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>288</v>
+        <v>403</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2651,7 +3011,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>290</v>
+        <v>404</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2743,7 +3103,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>291</v>
+        <v>407</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2835,7 +3195,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>296</v>
+        <v>412</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2927,7 +3287,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>298</v>
+        <v>414</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3019,7 +3379,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>297</v>
+        <v>413</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3477,7 +3837,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>272</v>
+        <v>388</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3759,7 +4119,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>299</v>
+        <v>415</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3851,7 +4211,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>300</v>
+        <v>417</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3943,7 +4303,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>301</v>
+        <v>418</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4035,7 +4395,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>302</v>
+        <v>419</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4127,7 +4487,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>303</v>
+        <v>420</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4219,7 +4579,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>304</v>
+        <v>421</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4314,7 +4674,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>316</v>
+        <v>435</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>25</v>
@@ -4411,7 +4771,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>313</v>
+        <v>432</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4503,7 +4863,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>305</v>
+        <v>422</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4598,7 +4958,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>294</v>
+        <v>410</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4690,7 +5050,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>279</v>
+        <v>395</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4785,7 +5145,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>276</v>
+        <v>391</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4877,7 +5237,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>319</v>
+        <v>439</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4969,7 +5329,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>323</v>
+        <v>444</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -5061,7 +5421,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>318</v>
+        <v>445</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -5153,7 +5513,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>325</v>
+        <v>441</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -5245,7 +5605,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>321</v>
+        <v>443</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>26</v>
@@ -5339,7 +5699,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>295</v>
+        <v>411</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -5431,7 +5791,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>277</v>
+        <v>393</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -5523,7 +5883,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>310</v>
+        <v>427</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -5615,7 +5975,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>280</v>
+        <v>396</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -5710,7 +6070,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>275</v>
+        <v>390</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -5802,7 +6162,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>278</v>
+        <v>394</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -5897,7 +6257,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>293</v>
+        <v>408</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -5992,7 +6352,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>309</v>
+        <v>426</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>

</xml_diff>

<commit_message>
IWP 2.5, 3.0 Demo
</commit_message>
<xml_diff>
--- a/KatalonData/BWPBootstrapData/BWPACHData.xlsx
+++ b/KatalonData/BWPBootstrapData/BWPACHData.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2679" uniqueCount="446">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3167" uniqueCount="568">
   <si>
     <t>Result</t>
   </si>
@@ -1412,6 +1412,372 @@
   </si>
   <si>
     <t>Thu May 07 21:00:28 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Jun 08 23:56:19 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Jun 08 23:56:54 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Jun 08 23:58:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Jun 08 23:58:48 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Jun 08 23:59:09 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:00:12 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:00:33 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:00:54 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:05:34 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:06:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:06:34 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:07:35 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:08:09 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:08:42 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:09:46 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:10:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:10:53 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:13:22 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:13:51 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:14:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:15:22 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:15:57 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:16:31 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:18:45 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:19:59 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:20:36 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:21:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:22:44 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:23:23 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:23:58 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:28:46 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:29:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:30:47 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:31:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:32:48 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:33:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:33:48 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:34:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:34:58 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:37:06 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:37:40 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:39:11 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:39:44 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:41:15 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:43:22 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:44:51 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:47:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:48:08 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:48:41 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:50:43 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:52:19 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:52:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:53:19 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:53:51 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:56:32 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:57:23 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:57:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:59:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 00:59:41 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:00:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:00:29 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:01:13 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:01:36 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:01:57 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:08:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:08:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:09:07 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:10:13 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:10:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:11:23 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:12:33 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:13:10 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:13:48 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:19:28 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:20:02 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:20:38 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:22:01 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:22:41 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:23:21 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:24:41 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:25:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:26:08 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:27:43 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:28:29 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:29:15 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:32:56 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:33:35 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:35:06 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:35:42 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:37:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:37:52 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:39:23 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:40:53 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:42:27 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:42:58 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:43:41 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:44:24 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:45:58 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:46:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:49:00 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:50:34 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:52:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:54:08 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:54:43 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:55:22 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:56:02 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:57:33 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 01:59:36 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 02:00:09 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 02:02:12 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 02:03:41 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 02:05:41 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 02:07:19 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 02:09:02 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 02:10:31 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 02:12:32 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 02:14:34 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 02:17:17 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 02:19:58 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 19:54:30 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 20:05:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 09 20:07:15 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -1805,7 +2171,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>423</v>
+        <v>533</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>23</v>
@@ -1905,7 +2271,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>429</v>
+        <v>543</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -1997,7 +2363,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>437</v>
+        <v>549</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2089,7 +2455,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>428</v>
+        <v>541</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2181,7 +2547,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>389</v>
+        <v>502</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2273,7 +2639,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>397</v>
+        <v>510</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2365,7 +2731,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>398</v>
+        <v>511</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2457,7 +2823,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>399</v>
+        <v>512</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2549,7 +2915,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>400</v>
+        <v>513</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2641,7 +3007,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>401</v>
+        <v>514</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2733,7 +3099,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>402</v>
+        <v>515</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2825,7 +3191,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>425</v>
+        <v>535</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>23</v>
@@ -2919,7 +3285,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>403</v>
+        <v>516</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3011,7 +3377,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>404</v>
+        <v>517</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3103,7 +3469,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>407</v>
+        <v>518</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3195,7 +3561,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>412</v>
+        <v>522</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3287,7 +3653,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>414</v>
+        <v>524</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3379,7 +3745,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>413</v>
+        <v>523</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -3837,7 +4203,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>388</v>
+        <v>501</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4119,7 +4485,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>415</v>
+        <v>525</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4211,7 +4577,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>417</v>
+        <v>526</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4303,7 +4669,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>418</v>
+        <v>527</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4395,7 +4761,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>419</v>
+        <v>528</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4487,7 +4853,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>420</v>
+        <v>529</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4579,7 +4945,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>421</v>
+        <v>530</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4674,7 +5040,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>435</v>
+        <v>548</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>25</v>
@@ -4771,7 +5137,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>432</v>
+        <v>565</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -4863,7 +5229,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>422</v>
+        <v>531</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -4958,7 +5324,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>410</v>
+        <v>520</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -5050,7 +5416,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>395</v>
+        <v>508</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -5145,7 +5511,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>391</v>
+        <v>505</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -5237,7 +5603,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>439</v>
+        <v>553</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -5329,7 +5695,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>444</v>
+        <v>564</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -5421,7 +5787,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>445</v>
+        <v>550</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -5513,7 +5879,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>441</v>
+        <v>566</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -5605,7 +5971,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>443</v>
+        <v>567</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>26</v>
@@ -5699,7 +6065,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>411</v>
+        <v>521</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -5791,7 +6157,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>393</v>
+        <v>506</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -5883,7 +6249,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>427</v>
+        <v>540</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -5975,7 +6341,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>396</v>
+        <v>509</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">
@@ -6070,7 +6436,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>390</v>
+        <v>504</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -6162,7 +6528,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>394</v>
+        <v>507</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -6257,7 +6623,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>408</v>
+        <v>519</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -6352,7 +6718,7 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>426</v>
+        <v>539</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>

</xml_diff>